<commit_message>
Enhance resident management with barangay association and bulk delete functionality. Update schema to include barangayId in Resident model and establish relationships. Introduce bulk delete API for residents, allowing authorized users to delete multiple residents at once. Modify ResidentsPage and ResidentTable components to support bulk delete actions and improve user experience with selection features. Update import functionality to ensure residents are correctly associated with barangays during import processes.
</commit_message>
<xml_diff>
--- a/public/resident-import-sample.xlsx
+++ b/public/resident-import-sample.xlsx
@@ -650,10 +650,10 @@
         <v/>
       </c>
       <c r="AN2" t="str">
-        <v/>
+        <v>001</v>
       </c>
       <c r="AO2" t="str">
-        <v/>
+        <v>Purok 1</v>
       </c>
       <c r="AP2" t="b">
         <v>0</v>
@@ -781,10 +781,10 @@
         <v/>
       </c>
       <c r="AN3" t="str">
-        <v/>
+        <v>001</v>
       </c>
       <c r="AO3" t="str">
-        <v/>
+        <v>Purok 2</v>
       </c>
       <c r="AP3" t="b">
         <v>0</v>
@@ -912,10 +912,10 @@
         <v/>
       </c>
       <c r="AN4" t="str">
-        <v/>
+        <v>001</v>
       </c>
       <c r="AO4" t="str">
-        <v/>
+        <v>Purok 1</v>
       </c>
       <c r="AP4" t="b">
         <v>0</v>
@@ -1043,10 +1043,10 @@
         <v/>
       </c>
       <c r="AN5" t="str">
-        <v/>
+        <v>001</v>
       </c>
       <c r="AO5" t="str">
-        <v/>
+        <v>Purok 2</v>
       </c>
       <c r="AP5" t="b">
         <v>0</v>
@@ -1174,10 +1174,10 @@
         <v/>
       </c>
       <c r="AN6" t="str">
-        <v/>
+        <v>001</v>
       </c>
       <c r="AO6" t="str">
-        <v/>
+        <v>Purok 1</v>
       </c>
       <c r="AP6" t="b">
         <v>0</v>
@@ -1305,10 +1305,10 @@
         <v/>
       </c>
       <c r="AN7" t="str">
-        <v/>
+        <v>001</v>
       </c>
       <c r="AO7" t="str">
-        <v/>
+        <v>Purok 2</v>
       </c>
       <c r="AP7" t="b">
         <v>0</v>
@@ -1436,10 +1436,10 @@
         <v/>
       </c>
       <c r="AN8" t="str">
-        <v/>
+        <v>001</v>
       </c>
       <c r="AO8" t="str">
-        <v/>
+        <v>Purok 1</v>
       </c>
       <c r="AP8" t="b">
         <v>0</v>
@@ -1567,10 +1567,10 @@
         <v/>
       </c>
       <c r="AN9" t="str">
-        <v/>
+        <v>001</v>
       </c>
       <c r="AO9" t="str">
-        <v/>
+        <v>Purok 2</v>
       </c>
       <c r="AP9" t="b">
         <v>0</v>
@@ -1698,10 +1698,10 @@
         <v/>
       </c>
       <c r="AN10" t="str">
-        <v/>
+        <v>001</v>
       </c>
       <c r="AO10" t="str">
-        <v/>
+        <v>Purok 1</v>
       </c>
       <c r="AP10" t="b">
         <v>0</v>
@@ -1829,10 +1829,10 @@
         <v/>
       </c>
       <c r="AN11" t="str">
-        <v/>
+        <v>001</v>
       </c>
       <c r="AO11" t="str">
-        <v/>
+        <v>Purok 2</v>
       </c>
       <c r="AP11" t="b">
         <v>0</v>
@@ -1960,10 +1960,10 @@
         <v/>
       </c>
       <c r="AN12" t="str">
-        <v/>
+        <v>001</v>
       </c>
       <c r="AO12" t="str">
-        <v/>
+        <v>Purok 1</v>
       </c>
       <c r="AP12" t="b">
         <v>0</v>
@@ -2091,10 +2091,10 @@
         <v/>
       </c>
       <c r="AN13" t="str">
-        <v/>
+        <v>001</v>
       </c>
       <c r="AO13" t="str">
-        <v/>
+        <v>Purok 2</v>
       </c>
       <c r="AP13" t="b">
         <v>0</v>
@@ -2222,10 +2222,10 @@
         <v/>
       </c>
       <c r="AN14" t="str">
-        <v/>
+        <v>001</v>
       </c>
       <c r="AO14" t="str">
-        <v/>
+        <v>Purok 1</v>
       </c>
       <c r="AP14" t="b">
         <v>0</v>
@@ -2353,10 +2353,10 @@
         <v/>
       </c>
       <c r="AN15" t="str">
-        <v/>
+        <v>001</v>
       </c>
       <c r="AO15" t="str">
-        <v/>
+        <v>Purok 2</v>
       </c>
       <c r="AP15" t="b">
         <v>0</v>
@@ -2484,10 +2484,10 @@
         <v/>
       </c>
       <c r="AN16" t="str">
-        <v/>
+        <v>001</v>
       </c>
       <c r="AO16" t="str">
-        <v/>
+        <v>Purok 1</v>
       </c>
       <c r="AP16" t="b">
         <v>0</v>
@@ -2615,10 +2615,10 @@
         <v/>
       </c>
       <c r="AN17" t="str">
-        <v/>
+        <v>001</v>
       </c>
       <c r="AO17" t="str">
-        <v/>
+        <v>Purok 2</v>
       </c>
       <c r="AP17" t="b">
         <v>0</v>
@@ -2746,10 +2746,10 @@
         <v/>
       </c>
       <c r="AN18" t="str">
-        <v/>
+        <v>001</v>
       </c>
       <c r="AO18" t="str">
-        <v/>
+        <v>Purok 1</v>
       </c>
       <c r="AP18" t="b">
         <v>0</v>
@@ -2877,10 +2877,10 @@
         <v/>
       </c>
       <c r="AN19" t="str">
-        <v/>
+        <v>001</v>
       </c>
       <c r="AO19" t="str">
-        <v/>
+        <v>Purok 2</v>
       </c>
       <c r="AP19" t="b">
         <v>0</v>
@@ -3008,10 +3008,10 @@
         <v/>
       </c>
       <c r="AN20" t="str">
-        <v/>
+        <v>001</v>
       </c>
       <c r="AO20" t="str">
-        <v/>
+        <v>Purok 1</v>
       </c>
       <c r="AP20" t="b">
         <v>0</v>
@@ -3139,10 +3139,10 @@
         <v/>
       </c>
       <c r="AN21" t="str">
-        <v/>
+        <v>001</v>
       </c>
       <c r="AO21" t="str">
-        <v/>
+        <v>Purok 2</v>
       </c>
       <c r="AP21" t="b">
         <v>0</v>
@@ -3270,10 +3270,10 @@
         <v/>
       </c>
       <c r="AN22" t="str">
-        <v/>
+        <v>001</v>
       </c>
       <c r="AO22" t="str">
-        <v/>
+        <v>Purok 1</v>
       </c>
       <c r="AP22" t="b">
         <v>0</v>
@@ -3401,10 +3401,10 @@
         <v/>
       </c>
       <c r="AN23" t="str">
-        <v/>
+        <v>001</v>
       </c>
       <c r="AO23" t="str">
-        <v/>
+        <v>Purok 2</v>
       </c>
       <c r="AP23" t="b">
         <v>0</v>
@@ -3532,10 +3532,10 @@
         <v/>
       </c>
       <c r="AN24" t="str">
-        <v/>
+        <v>001</v>
       </c>
       <c r="AO24" t="str">
-        <v/>
+        <v>Purok 1</v>
       </c>
       <c r="AP24" t="b">
         <v>0</v>
@@ -3663,10 +3663,10 @@
         <v/>
       </c>
       <c r="AN25" t="str">
-        <v/>
+        <v>001</v>
       </c>
       <c r="AO25" t="str">
-        <v/>
+        <v>Purok 2</v>
       </c>
       <c r="AP25" t="b">
         <v>0</v>
@@ -3794,10 +3794,10 @@
         <v/>
       </c>
       <c r="AN26" t="str">
-        <v/>
+        <v>001</v>
       </c>
       <c r="AO26" t="str">
-        <v/>
+        <v>Purok 1</v>
       </c>
       <c r="AP26" t="b">
         <v>0</v>
@@ -3925,10 +3925,10 @@
         <v/>
       </c>
       <c r="AN27" t="str">
-        <v/>
+        <v>001</v>
       </c>
       <c r="AO27" t="str">
-        <v/>
+        <v>Purok 2</v>
       </c>
       <c r="AP27" t="b">
         <v>0</v>
@@ -4056,10 +4056,10 @@
         <v/>
       </c>
       <c r="AN28" t="str">
-        <v/>
+        <v>001</v>
       </c>
       <c r="AO28" t="str">
-        <v/>
+        <v>Purok 1</v>
       </c>
       <c r="AP28" t="b">
         <v>0</v>
@@ -4187,10 +4187,10 @@
         <v/>
       </c>
       <c r="AN29" t="str">
-        <v/>
+        <v>001</v>
       </c>
       <c r="AO29" t="str">
-        <v/>
+        <v>Purok 2</v>
       </c>
       <c r="AP29" t="b">
         <v>0</v>
@@ -4318,10 +4318,10 @@
         <v/>
       </c>
       <c r="AN30" t="str">
-        <v/>
+        <v>001</v>
       </c>
       <c r="AO30" t="str">
-        <v/>
+        <v>Purok 1</v>
       </c>
       <c r="AP30" t="b">
         <v>0</v>
@@ -4449,10 +4449,10 @@
         <v/>
       </c>
       <c r="AN31" t="str">
-        <v/>
+        <v>001</v>
       </c>
       <c r="AO31" t="str">
-        <v/>
+        <v>Purok 2</v>
       </c>
       <c r="AP31" t="b">
         <v>0</v>
@@ -4470,7 +4470,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:A10"/>
+  <dimension ref="A1:A11"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -4504,27 +4504,32 @@
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>household_house_no + household_purok_name: must match existing household (exact purok name), or leave both empty.</v>
+        <v>household_house_no + household_purok_name: REQUIRED — must match an existing household (purok name exactly as in Settings → Puroks).</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>Booleans: TRUE/FALSE, Yes/No, 1/0</v>
+        <v>Sample rows: rows 2,4,6,… → house 001 + Purok 1; rows 3,5,7,… → 001 + Purok 2. Create those 2 households (Households → Add) before importing — puroks alone are not enough.</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>sss_no = SSS (Social Security System) number; aliases sss_no / sss accepted.</v>
+        <v>Booleans: TRUE/FALSE, Yes/No, 1/0</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
+        <v>sss_no = SSS (Social Security System) number; aliases sss_no / sss accepted.</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:A10"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:A11"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>